<commit_message>
Redesign the relative-interest deck
Rebuild Relative_Interest_Pie_Chart.pptx as a six-slide presentation with
a navy and orange theme, slide layouts with the footer and slide numbers,
sections and speaker notes. Each programme keeps one colour and icon on
every slide. The slides are the title, how the data was collected, the
pie chart with a headline figure and a key, what the chart shows, three
recommendations, and a closing slide.

The pie slices use a colour palette that passes a colour-blindness check
and carries white labels. The Excel pie chart now uses the same colours
and labels. The deck's figures are read from the finished workbook.

finish_deck.py can now add a Fade transition instead of Push
(--transition fade). Push stays the default for the other decks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WToQxHdrdWhM7bKqXvUa59
</commit_message>
<xml_diff>
--- a/assignment/Relative_Interest_Pie_Chart.xlsx
+++ b/assignment/Relative_Interest_Pie_Chart.xlsx
@@ -251,10 +251,10 @@
           <yMode val="edge"/>
           <wMode val="factor"/>
           <hMode val="factor"/>
-          <x val="0.07000000000000001"/>
-          <y val="0.2"/>
-          <w val="0.42"/>
-          <h val="0.7"/>
+          <x val="0.06"/>
+          <y val="0.17"/>
+          <w val="0.46"/>
+          <h val="0.78"/>
         </manualLayout>
       </layout>
       <pieChart>
@@ -276,13 +276,11 @@
             <idx val="0"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="75000"/>
-                </a:schemeClr>
+                <a:srgbClr val="C55A11"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
-                  <a:schemeClr val="bg1"/>
+                  <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -292,13 +290,11 @@
             <idx val="1"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="50000"/>
-                </a:schemeClr>
+                <a:srgbClr val="2A78D6"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
-                  <a:schemeClr val="bg1"/>
+                  <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -308,13 +304,11 @@
             <idx val="2"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="75000"/>
-                </a:schemeClr>
+                <a:srgbClr val="0F8A5F"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
-                  <a:schemeClr val="bg1"/>
+                  <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -324,11 +318,11 @@
             <idx val="3"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:schemeClr val="accent1"/>
+                <a:srgbClr val="4A3AA7"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
-                  <a:schemeClr val="bg1"/>
+                  <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -338,14 +332,11 @@
             <idx val="4"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="60000"/>
-                  <a:lumOff val="40000"/>
-                </a:schemeClr>
+                <a:srgbClr val="B03A8C"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
-                  <a:schemeClr val="bg1"/>
+                  <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -367,9 +358,9 @@
             <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
             <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:pPr>
-                <a:defRPr sz="1000" b="1">
+                <a:defRPr sz="1100" b="1">
                   <a:solidFill>
-                    <a:srgbClr val="404040"/>
+                    <a:srgbClr val="FFFFFF"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                 </a:defRPr>
@@ -377,23 +368,21 @@
               <a:r>
                 <a:t/>
               </a:r>
-              <a:endParaRPr sz="1000" b="1">
+              <a:endParaRPr sz="1100" b="1">
                 <a:solidFill>
-                  <a:srgbClr val="404040"/>
+                  <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
               </a:endParaRPr>
             </a:p>
           </txPr>
-          <dLblPos val="outEnd"/>
+          <dLblPos val="inEnd"/>
           <showLegendKey val="0"/>
-          <showVal val="1"/>
+          <showVal val="0"/>
           <showCatName val="0"/>
           <showSerName val="0"/>
           <showPercent val="1"/>
-          <separator>
-</separator>
-          <showLeaderLines val="1"/>
+          <showLeaderLines val="0"/>
         </dLbls>
         <firstSliceAng val="0"/>
       </pieChart>

</xml_diff>

<commit_message>
Make the pie chart deck plain black and white, with transitions
Replace the designed six-slide deck with a short, plain one on
PowerPoint 2013's standard layouts. The five slides are the title, the
table of scores, the pie chart, the observations and a thank-you slide.
The first and last slides are black with white text, the rest black on
white. The pie chart and its Excel workbook are now in black and greys.

Each slide gets its own transition: Fade, Push, Wipe, Split and Cover.
finish_deck.py now takes a comma-separated list of transitions and
knows Wipe, Split and Cover. Push stays the default for the other decks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WToQxHdrdWhM7bKqXvUa59
</commit_message>
<xml_diff>
--- a/assignment/Relative_Interest_Pie_Chart.xlsx
+++ b/assignment/Relative_Interest_Pie_Chart.xlsx
@@ -29,7 +29,7 @@
       <name val="Calibri"/>
       <family val="2"/>
       <b val="1"/>
-      <color theme="4" tint="-0.499984740745262"/>
+      <color theme="1"/>
       <sz val="14"/>
       <scheme val="minor"/>
     </font>
@@ -75,7 +75,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="-0.499984740745262"/>
+        <fgColor theme="1"/>
       </patternFill>
     </fill>
   </fills>
@@ -251,10 +251,10 @@
           <yMode val="edge"/>
           <wMode val="factor"/>
           <hMode val="factor"/>
-          <x val="0.06"/>
-          <y val="0.17"/>
-          <w val="0.46"/>
-          <h val="0.78"/>
+          <x val="0.09"/>
+          <y val="0.21"/>
+          <w val="0.41"/>
+          <h val="0.7"/>
         </manualLayout>
       </layout>
       <pieChart>
@@ -276,7 +276,7 @@
             <idx val="0"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="C55A11"/>
+                <a:srgbClr val="000000"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
@@ -290,7 +290,7 @@
             <idx val="1"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2A78D6"/>
+                <a:srgbClr val="404040"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
@@ -304,7 +304,7 @@
             <idx val="2"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="0F8A5F"/>
+                <a:srgbClr val="7F7F7F"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
@@ -318,7 +318,7 @@
             <idx val="3"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="4A3AA7"/>
+                <a:srgbClr val="A6A6A6"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
@@ -332,7 +332,7 @@
             <idx val="4"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="B03A8C"/>
+                <a:srgbClr val="D9D9D9"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
@@ -360,7 +360,7 @@
               <a:pPr>
                 <a:defRPr sz="1100" b="1">
                   <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
+                    <a:srgbClr val="000000"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                 </a:defRPr>
@@ -370,19 +370,19 @@
               </a:r>
               <a:endParaRPr sz="1100" b="1">
                 <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
+                  <a:srgbClr val="000000"/>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
               </a:endParaRPr>
             </a:p>
           </txPr>
-          <dLblPos val="inEnd"/>
+          <dLblPos val="outEnd"/>
           <showLegendKey val="0"/>
           <showVal val="0"/>
           <showCatName val="0"/>
           <showSerName val="0"/>
           <showPercent val="1"/>
-          <showLeaderLines val="0"/>
+          <showLeaderLines val="1"/>
         </dLbls>
         <firstSliceAng val="0"/>
       </pieChart>

</xml_diff>

<commit_message>
Give the pie chart deck three colour palettes
Build the relative-interest deck in three versions with the same five
plain slides and transitions:

- Marketing: the Marketing Budget deck's palette (Arial, dark-blue titles
  over a line, a thin light-blue frame, light-blue boxes, grey pie).
- PZ: the PZ Nigeria deck's wood design (wood background, white cards
  with an orange border, straps on the title slides, Rockwell type,
  orange-brown accents, a brown and orange pie).
- Mixed: wood title slides with dark-blue and orange content slides.

Each deck's theme carries its colours and fonts. make_wood.py draws the
wood background. The Excel pie chart now orders its greys like the
Marketing Budget deck's.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WToQxHdrdWhM7bKqXvUa59
</commit_message>
<xml_diff>
--- a/assignment/Relative_Interest_Pie_Chart.xlsx
+++ b/assignment/Relative_Interest_Pie_Chart.xlsx
@@ -276,7 +276,7 @@
             <idx val="0"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="000000"/>
+                <a:srgbClr val="262626"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
@@ -290,7 +290,7 @@
             <idx val="1"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="404040"/>
+                <a:srgbClr val="A6A6A6"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
@@ -304,7 +304,7 @@
             <idx val="2"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="7F7F7F"/>
+                <a:srgbClr val="595959"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
@@ -318,7 +318,7 @@
             <idx val="3"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="A6A6A6"/>
+                <a:srgbClr val="D9D9D9"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>
@@ -332,7 +332,7 @@
             <idx val="4"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="D9D9D9"/>
+                <a:srgbClr val="7F7F7F"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
                 <a:solidFill>

</xml_diff>